<commit_message>
Add digikey part numbers
</commit_message>
<xml_diff>
--- a/15W-Receiver/BOM/15W-Receiver.xlsx
+++ b/15W-Receiver/BOM/15W-Receiver.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\farvisionsystems\stelon-qiwirelesscharger\Design-Files\15W-Receiver\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\Qi Wireless charger\QI-Wireless-Charger-Boards\15W-Receiver\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC112537-F55F-48C0-92BA-776BE5640BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="305">
   <si>
     <t>#</t>
   </si>
@@ -273,30 +272,12 @@
     <t>J1</t>
   </si>
   <si>
-    <t>Gold 250V 3A Straight Square Pins 2.5mm 5P 260℃ 6mm -40℃~+105℃ 3mm 2.54mm Plugin Black Brass 1x5P Plugin,P=2.54mm Pin Headers ROHS</t>
-  </si>
-  <si>
-    <t>HDR1X5_</t>
-  </si>
-  <si>
-    <t>X6511WV-05H-C60D30</t>
-  </si>
-  <si>
     <t>XKB</t>
   </si>
   <si>
     <t>J2</t>
   </si>
   <si>
-    <t>Gold 250V 3A Straight Square Pins 2.5mm 4P 260℃ 6mm -40℃~+105℃ 3mm 2.54mm Plugin Black Brass 1x4P Plugin,P=2.54mm Pin Headers ROHS</t>
-  </si>
-  <si>
-    <t>HDR1X4_</t>
-  </si>
-  <si>
-    <t>X6511WV-04H-C60D30</t>
-  </si>
-  <si>
     <t>Inductor</t>
   </si>
   <si>
@@ -399,9 +380,6 @@
     <t>MMBT3904</t>
   </si>
   <si>
-    <t>ElecSuper</t>
-  </si>
-  <si>
     <t>Q8</t>
   </si>
   <si>
@@ -483,12 +461,6 @@
     <t>R8</t>
   </si>
   <si>
-    <t>ERJ-3EKF1102V - RES TKF 11k 1% 1/10W SMD 0603</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF1102V</t>
-  </si>
-  <si>
     <t>Panasonic Electronic Components</t>
   </si>
   <si>
@@ -498,12 +470,6 @@
     <t>R9, R12</t>
   </si>
   <si>
-    <t>ERJ3EKF10R0V - RES TKF 10R 1% 1/10W SMD 0603, RC0603FR-0710RL - 10R 0603</t>
-  </si>
-  <si>
-    <t>ERJ3EKF10R0V</t>
-  </si>
-  <si>
     <t>10R</t>
   </si>
   <si>
@@ -774,15 +740,6 @@
     <t>R5, R7, R24, R25, R31</t>
   </si>
   <si>
-    <t>MC0063W060311K</t>
-  </si>
-  <si>
-    <t>Multicomp</t>
-  </si>
-  <si>
-    <t>MC0063W060311K - RES TKF 1k 1% 1/16W SMD 0603</t>
-  </si>
-  <si>
     <t>RES TKF 1k 1% 1/10W SMD 060</t>
   </si>
   <si>
@@ -805,13 +762,200 @@
   </si>
   <si>
     <t>RES 4.7kΩ ±5% 100mW 0603</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Supplier Part Number</t>
+  </si>
+  <si>
+    <t>311-1488-1-ND</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>399-C0805C473K5RACTUCT-ND</t>
+  </si>
+  <si>
+    <t>399-C0603C680J1GACTUCT-ND</t>
+  </si>
+  <si>
+    <t>732-7583-1-ND</t>
+  </si>
+  <si>
+    <t>311-1802-1-ND</t>
+  </si>
+  <si>
+    <t>587-3166-1-ND</t>
+  </si>
+  <si>
+    <t>4988-NMC0603X7R102K50TRPFCT-ND</t>
+  </si>
+  <si>
+    <t>445-7631-1-ND</t>
+  </si>
+  <si>
+    <t>478-KGM15BR71E104JTCT-ND</t>
+  </si>
+  <si>
+    <t>1276-1005-1-ND</t>
+  </si>
+  <si>
+    <t>732-7968-1-ND</t>
+  </si>
+  <si>
+    <t>1727-1350-1-ND</t>
+  </si>
+  <si>
+    <t>475-LRTBR48G-P9Q7-1+R7S5-26+NP-68-R33-ZBCT-ND</t>
+  </si>
+  <si>
+    <t>497-7163-1-ND</t>
+  </si>
+  <si>
+    <t>MBR120VLSFT3GOSCT-ND</t>
+  </si>
+  <si>
+    <t>732-5318-ND</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole 5 position 0.100" (2.54mm)</t>
+  </si>
+  <si>
+    <t>732-5317-ND</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole 4 position 0.100" (2.54mm)</t>
+  </si>
+  <si>
+    <t>732-6209-ND</t>
+  </si>
+  <si>
+    <t>2457-XAL6060-153MEC-ND</t>
+  </si>
+  <si>
+    <t>2N7002-FDICT-ND</t>
+  </si>
+  <si>
+    <t>SI4816BDY-T1-E3CT-ND</t>
+  </si>
+  <si>
+    <t>SI3433CDV-T1-GE3CT-ND</t>
+  </si>
+  <si>
+    <t>785-1306-1-ND</t>
+  </si>
+  <si>
+    <t>4786-MMBT3904CT-ND</t>
+  </si>
+  <si>
+    <t>Good-Ark Semiconductor</t>
+  </si>
+  <si>
+    <t>DMG3415UDICT-ND</t>
+  </si>
+  <si>
+    <t>311-5.10KHRCT-ND</t>
+  </si>
+  <si>
+    <t>A102203CT-ND</t>
+  </si>
+  <si>
+    <t>RMCF0603FT1K00CT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 
+1 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>541-11.3KHCT-ND</t>
+  </si>
+  <si>
+    <t>RMCF0603FT11K0CT-ND</t>
+  </si>
+  <si>
+    <t>RMCF0603FT11K0</t>
+  </si>
+  <si>
+    <t>11 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>10 Ohms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>RMCF0603FT10R0</t>
+  </si>
+  <si>
+    <t>RMCF0603FT10R0CT-ND</t>
+  </si>
+  <si>
+    <t>P220KHCT-ND</t>
+  </si>
+  <si>
+    <t>311-20.0KHRCT-ND</t>
+  </si>
+  <si>
+    <t>541-510HCT-ND</t>
+  </si>
+  <si>
+    <t>WSLP-.05CT-ND</t>
+  </si>
+  <si>
+    <t>CRA2512-FZ-R100ELFCT-ND</t>
+  </si>
+  <si>
+    <t>311-68GRCT-ND</t>
+  </si>
+  <si>
+    <t>311-270GRCT-ND</t>
+  </si>
+  <si>
+    <t>311-4.7KGRCT-ND</t>
+  </si>
+  <si>
+    <t>311-0.0GRCT-ND</t>
+  </si>
+  <si>
+    <t>4809-SKRPABE010CT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SW1020CT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 150-MCP1799T-5002H/TTCT-ND</t>
+  </si>
+  <si>
+    <t>PIC16F18345-E/GZ-ND</t>
+  </si>
+  <si>
+    <t>AP2127K-3.3TRG1DICT-ND</t>
+  </si>
+  <si>
+    <t>MCP6021T-E/OTCT-ND</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>579-MCP14628-E/SN</t>
+  </si>
+  <si>
+    <t>296-27898-1-ND</t>
+  </si>
+  <si>
+    <t>MAX17048G+T10CT-ND</t>
+  </si>
+  <si>
+    <t>497-STM32G030F6P6-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -854,6 +998,33 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -875,7 +1046,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -966,11 +1137,104 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1007,15 +1271,55 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1296,24 +1600,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M54"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" customWidth="1"/>
-    <col min="9" max="9" width="17.88671875" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="9" width="21.42578125" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1322,11 +1627,13 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" thickBot="1">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1349,17 +1656,23 @@
       <c r="H2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="J2" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="24">
+    <row r="3" spans="1:13" ht="24.75" thickBot="1">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
         <f>ROW(B3)-ROW($B$2)</f>
@@ -1371,7 +1684,7 @@
       <c r="D3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="23" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -1383,15 +1696,21 @@
       <c r="H3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="K3" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="9">
+      <c r="L3" s="9">
         <v>2</v>
       </c>
-      <c r="K3" s="9"/>
-    </row>
-    <row r="4" spans="1:11" ht="24">
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" spans="1:13" ht="24.75" thickBot="1">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
         <f t="shared" ref="B4:B54" si="0">ROW(B4)-ROW($B$2)</f>
@@ -1401,9 +1720,9 @@
         <v>10</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="E4" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="11" t="s">
@@ -1415,15 +1734,21 @@
       <c r="H4" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="K4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="11">
+      <c r="L4" s="11">
         <v>2</v>
       </c>
-      <c r="K4" s="11"/>
-    </row>
-    <row r="5" spans="1:11" ht="24">
+      <c r="M4" s="11"/>
+    </row>
+    <row r="5" spans="1:13" ht="24.75" thickBot="1">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
         <f t="shared" si="0"/>
@@ -1441,21 +1766,27 @@
       <c r="F5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="28" t="s">
         <v>24</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="K5" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="9">
+      <c r="L5" s="9">
         <v>1</v>
       </c>
-      <c r="K5" s="9"/>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickBot="1">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
         <f t="shared" si="0"/>
@@ -1468,26 +1799,32 @@
         <v>27</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>234</v>
+      <c r="G6" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="K6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="11">
+      <c r="L6" s="11">
         <v>3</v>
       </c>
-      <c r="K6" s="11"/>
-    </row>
-    <row r="7" spans="1:11" ht="24">
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" spans="1:13" ht="24.75" thickBot="1">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f t="shared" si="0"/>
@@ -1505,21 +1842,27 @@
       <c r="F7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="23" t="s">
         <v>33</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="K7" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="9">
+      <c r="L7" s="9">
         <v>6</v>
       </c>
-      <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="1:11" ht="24">
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" spans="1:13" ht="24.75" thickBot="1">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
         <f t="shared" si="0"/>
@@ -1531,7 +1874,7 @@
       <c r="D8" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="25" t="s">
         <v>37</v>
       </c>
       <c r="F8" s="11" t="s">
@@ -1543,15 +1886,21 @@
       <c r="H8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="K8" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="11">
+      <c r="L8" s="11">
         <v>2</v>
       </c>
-      <c r="K8" s="11"/>
-    </row>
-    <row r="9" spans="1:11" ht="24">
+      <c r="M8" s="11"/>
+    </row>
+    <row r="9" spans="1:13" ht="36.75" thickBot="1">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
         <f t="shared" si="0"/>
@@ -1563,7 +1912,7 @@
       <c r="D9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="23" t="s">
         <v>41</v>
       </c>
       <c r="F9" s="9" t="s">
@@ -1575,15 +1924,21 @@
       <c r="H9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="K9" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="J9" s="9">
+      <c r="L9" s="9">
         <v>2</v>
       </c>
-      <c r="K9" s="9"/>
-    </row>
-    <row r="10" spans="1:11" ht="24.6" thickBot="1">
+      <c r="M9" s="9"/>
+    </row>
+    <row r="10" spans="1:13" ht="24.75" thickBot="1">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
         <f t="shared" si="0"/>
@@ -1595,7 +1950,7 @@
       <c r="D10" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="25" t="s">
         <v>46</v>
       </c>
       <c r="F10" s="11" t="s">
@@ -1607,44 +1962,56 @@
       <c r="H10" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K10" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="J10" s="11">
+      <c r="L10" s="11">
         <v>2</v>
       </c>
-      <c r="K10" s="11"/>
-    </row>
-    <row r="11" spans="1:11" ht="15" thickBot="1">
+      <c r="M10" s="11"/>
+    </row>
+    <row r="11" spans="1:13" ht="24.75" thickBot="1">
       <c r="A11" s="2"/>
       <c r="B11" s="7"/>
       <c r="C11" s="8" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="23" t="s">
         <v>50</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="K11" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="9">
+      <c r="L11" s="9">
         <v>3</v>
       </c>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1">
+      <c r="M11" s="9"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
         <f t="shared" si="0"/>
@@ -1654,29 +2021,35 @@
         <v>10</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>240</v>
+      <c r="G12" s="23" t="s">
+        <v>229</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="I12" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="I12" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J12" s="26" t="s">
+        <v>255</v>
+      </c>
+      <c r="K12" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="9">
+      <c r="L12" s="9">
         <v>5</v>
       </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="24.6" thickBot="1">
+      <c r="M12" s="9"/>
+    </row>
+    <row r="13" spans="1:13" ht="24.75" thickBot="1">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
         <f t="shared" si="0"/>
@@ -1694,21 +2067,27 @@
       <c r="F13" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="G13" s="29" t="s">
         <v>54</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J13" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="K13" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="J13" s="11">
+      <c r="L13" s="11">
         <v>1</v>
       </c>
-      <c r="K13" s="11"/>
-    </row>
-    <row r="14" spans="1:11" ht="24">
+      <c r="M13" s="11"/>
+    </row>
+    <row r="14" spans="1:13" ht="24.75" thickBot="1">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
         <f t="shared" si="0"/>
@@ -1726,21 +2105,27 @@
       <c r="F14" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="23" t="s">
         <v>60</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J14" s="26" t="s">
+        <v>257</v>
+      </c>
+      <c r="K14" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J14" s="9">
+      <c r="L14" s="9">
         <v>4</v>
       </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="48">
+      <c r="M14" s="9"/>
+    </row>
+    <row r="15" spans="1:13" ht="48.75" thickBot="1">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
         <f t="shared" si="0"/>
@@ -1758,21 +2143,27 @@
       <c r="F15" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="25" t="s">
         <v>65</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="I15" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J15" s="27" t="s">
+        <v>258</v>
+      </c>
+      <c r="K15" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J15" s="11">
+      <c r="L15" s="11">
         <v>1</v>
       </c>
-      <c r="K15" s="11"/>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="M15" s="11"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
         <f t="shared" si="0"/>
@@ -1790,21 +2181,27 @@
       <c r="F16" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="23" t="s">
         <v>70</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="I16" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J16" s="26" t="s">
+        <v>259</v>
+      </c>
+      <c r="K16" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J16" s="9">
+      <c r="L16" s="9">
         <v>1</v>
       </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="M16" s="9"/>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" thickBot="1">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
         <f t="shared" si="0"/>
@@ -1822,21 +2219,27 @@
       <c r="F17" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="25" t="s">
         <v>75</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="I17" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J17" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="K17" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J17" s="11">
+      <c r="L17" s="11">
         <v>1</v>
       </c>
-      <c r="K17" s="11"/>
-    </row>
-    <row r="18" spans="1:11" ht="48">
+      <c r="M17" s="11"/>
+    </row>
+    <row r="18" spans="1:13" ht="24.75" thickBot="1">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
         <f t="shared" si="0"/>
@@ -1848,27 +2251,33 @@
       <c r="D18" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="E18" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="23">
+        <v>61300511121</v>
+      </c>
+      <c r="H18" s="9">
+        <v>61300511121</v>
+      </c>
+      <c r="I18" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="K18" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J18" s="9">
+      <c r="L18" s="9">
         <v>1</v>
       </c>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="48">
+      <c r="M18" s="9"/>
+    </row>
+    <row r="19" spans="1:13" ht="24.75" thickBot="1">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
         <f t="shared" si="0"/>
@@ -1878,1150 +2287,1366 @@
         <v>77</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>86</v>
+        <v>264</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="25">
+        <v>61300411121</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="I19" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="K19" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J19" s="11">
+      <c r="L19" s="11">
         <v>1</v>
       </c>
-      <c r="K19" s="11"/>
-    </row>
-    <row r="20" spans="1:11" ht="24">
+      <c r="M19" s="11"/>
+    </row>
+    <row r="20" spans="1:13" ht="24.75" thickBot="1">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G20" s="10" t="s">
-        <v>90</v>
+      <c r="G20" s="23" t="s">
+        <v>84</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J20" s="9">
+        <v>85</v>
+      </c>
+      <c r="I20" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="L20" s="9">
         <v>1</v>
       </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="M20" s="9"/>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" thickBot="1">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D21" s="11" t="s">
-        <v>93</v>
-      </c>
       <c r="E21" s="12" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>96</v>
+        <v>89</v>
+      </c>
+      <c r="G21" s="29" t="s">
+        <v>90</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="I21" s="12" t="s">
+      <c r="I21" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="K21" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J21" s="11">
+      <c r="L21" s="11">
         <v>1</v>
       </c>
-      <c r="K21" s="11"/>
-    </row>
-    <row r="22" spans="1:11" ht="24">
+      <c r="M21" s="11"/>
+    </row>
+    <row r="22" spans="1:13" ht="24.75" thickBot="1">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>101</v>
+        <v>94</v>
+      </c>
+      <c r="G22" s="23" t="s">
+        <v>95</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="I22" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="I22" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="K22" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J22" s="9">
+      <c r="L22" s="9">
         <v>3</v>
       </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="24">
+      <c r="M22" s="9"/>
+    </row>
+    <row r="23" spans="1:13" ht="24.75" thickBot="1">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="11" t="s">
-        <v>103</v>
-      </c>
       <c r="E23" s="12" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>106</v>
+        <v>99</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>100</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="I23" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="I23" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J23" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="K23" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J23" s="11">
+      <c r="L23" s="11">
         <v>1</v>
       </c>
-      <c r="K23" s="11"/>
-    </row>
-    <row r="24" spans="1:11" ht="24">
+      <c r="M23" s="11"/>
+    </row>
+    <row r="24" spans="1:13" ht="24.75" thickBot="1">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>111</v>
+        <v>104</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>105</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="I24" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="I24" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="K24" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J24" s="9">
+      <c r="L24" s="9">
         <v>1</v>
       </c>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" ht="36">
+      <c r="M24" s="9"/>
+    </row>
+    <row r="25" spans="1:13" ht="36.75" thickBot="1">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="G25" s="12" t="s">
-        <v>114</v>
+      <c r="G25" s="25" t="s">
+        <v>108</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="I25" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I25" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="K25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J25" s="11">
+      <c r="L25" s="11">
         <v>1</v>
       </c>
-      <c r="K25" s="11"/>
-    </row>
-    <row r="26" spans="1:11" ht="24">
+      <c r="M25" s="11"/>
+    </row>
+    <row r="26" spans="1:13" ht="24.75" thickBot="1">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>120</v>
+        <v>113</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>114</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="I26" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="I26" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="K26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J26" s="9">
+      <c r="L26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11">
+      <c r="M26" s="9"/>
+    </row>
+    <row r="27" spans="1:13" ht="15.75" thickBot="1">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="G27" s="12" t="s">
-        <v>124</v>
+        <v>113</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>117</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="I27" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="I27" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="K27" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J27" s="11">
+      <c r="L27" s="11">
         <v>1</v>
       </c>
-      <c r="K27" s="11"/>
-    </row>
-    <row r="28" spans="1:11" ht="24">
+      <c r="M27" s="11"/>
+    </row>
+    <row r="28" spans="1:13" ht="24.75" thickBot="1">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>130</v>
+        <v>122</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>123</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="J28" s="9">
+        <v>124</v>
+      </c>
+      <c r="I28" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="L28" s="9">
         <v>1</v>
       </c>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11">
+      <c r="M28" s="9"/>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" thickBot="1">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>133</v>
-      </c>
       <c r="E29" s="12" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G29" s="12" t="s">
-        <v>242</v>
+        <v>127</v>
+      </c>
+      <c r="G29" s="25" t="s">
+        <v>231</v>
       </c>
       <c r="H29" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I29" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="J29" s="11">
+      <c r="I29" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J29" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="L29" s="11">
         <v>1</v>
       </c>
-      <c r="K29" s="11"/>
-    </row>
-    <row r="30" spans="1:11" ht="24">
+      <c r="M29" s="11"/>
+    </row>
+    <row r="30" spans="1:13" ht="24.75" thickBot="1">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>138</v>
+        <v>127</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>131</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="J30" s="9">
+        <v>132</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J30" s="26" t="s">
+        <v>275</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="L30" s="9">
         <v>10</v>
       </c>
-      <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" ht="24.6" thickBot="1">
+      <c r="M30" s="9"/>
+    </row>
+    <row r="31" spans="1:13" ht="48.75" thickBot="1">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="E31" s="12" t="s">
-        <v>248</v>
+        <v>234</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>277</v>
       </c>
       <c r="F31" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="G31" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="G31" s="12" t="s">
-        <v>246</v>
-      </c>
       <c r="H31" s="11" t="s">
-        <v>247</v>
-      </c>
-      <c r="I31" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J31" s="11">
+        <v>135</v>
+      </c>
+      <c r="I31" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J31" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="K31" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="L31" s="11">
         <v>5</v>
       </c>
-      <c r="K31" s="11"/>
-    </row>
-    <row r="32" spans="1:11" ht="15" thickBot="1">
+      <c r="M31" s="11"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" thickBot="1">
       <c r="A32" s="2"/>
       <c r="B32" s="7"/>
       <c r="C32" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="F32" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="G32" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="G32" s="12" t="s">
-        <v>141</v>
-      </c>
       <c r="H32" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="I32" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J32" s="9">
+        <v>135</v>
+      </c>
+      <c r="I32" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J32" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="L32" s="9">
         <v>1</v>
       </c>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" ht="24.6" thickBot="1">
+      <c r="M32" s="9"/>
+    </row>
+    <row r="33" spans="1:13" ht="24.75" thickBot="1">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="J33" s="9">
+        <v>124</v>
+      </c>
+      <c r="I33" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J33" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="L33" s="9">
         <v>1</v>
       </c>
-      <c r="K33" s="9"/>
-    </row>
-    <row r="34" spans="1:11" ht="24">
+      <c r="M33" s="9"/>
+    </row>
+    <row r="34" spans="1:13" ht="36.75" thickBot="1">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>149</v>
+        <v>281</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G34" s="12" t="s">
-        <v>150</v>
+        <v>127</v>
+      </c>
+      <c r="G34" s="25" t="s">
+        <v>280</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="I34" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="J34" s="11">
+        <v>135</v>
+      </c>
+      <c r="I34" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J34" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="K34" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="L34" s="11">
         <v>1</v>
       </c>
-      <c r="K34" s="11"/>
-    </row>
-    <row r="35" spans="1:11" ht="24">
+      <c r="M34" s="11"/>
+    </row>
+    <row r="35" spans="1:13" ht="36.75" thickBot="1">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>154</v>
+        <v>282</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>155</v>
+        <v>127</v>
+      </c>
+      <c r="G35" s="23" t="s">
+        <v>283</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="I35" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="J35" s="9">
+        <v>135</v>
+      </c>
+      <c r="I35" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J35" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="L35" s="9">
         <v>2</v>
       </c>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" ht="24">
+      <c r="M35" s="9"/>
+    </row>
+    <row r="36" spans="1:13" ht="24.75" thickBot="1">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>159</v>
+        <v>127</v>
+      </c>
+      <c r="G36" s="25" t="s">
+        <v>148</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="I36" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="J36" s="11">
+        <v>142</v>
+      </c>
+      <c r="I36" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J36" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="L36" s="11">
         <v>2</v>
       </c>
-      <c r="K36" s="11"/>
-    </row>
-    <row r="37" spans="1:11" ht="24">
+      <c r="M36" s="11"/>
+    </row>
+    <row r="37" spans="1:13" ht="24.75" thickBot="1">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>163</v>
+        <v>127</v>
+      </c>
+      <c r="G37" s="23" t="s">
+        <v>152</v>
       </c>
       <c r="H37" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I37" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="J37" s="9">
+      <c r="I37" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J37" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="L37" s="9">
         <v>3</v>
       </c>
-      <c r="K37" s="9"/>
-    </row>
-    <row r="38" spans="1:11" ht="24">
+      <c r="M37" s="9"/>
+    </row>
+    <row r="38" spans="1:13" ht="24.75" thickBot="1">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>167</v>
+        <v>127</v>
+      </c>
+      <c r="G38" s="25" t="s">
+        <v>156</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="J38" s="11">
+        <v>124</v>
+      </c>
+      <c r="I38" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J38" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="K38" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="L38" s="11">
         <v>2</v>
       </c>
-      <c r="K38" s="11"/>
-    </row>
-    <row r="39" spans="1:11" ht="24">
+      <c r="M38" s="11"/>
+    </row>
+    <row r="39" spans="1:13" ht="24.75" thickBot="1">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="G39" s="10" t="s">
-        <v>171</v>
+        <v>122</v>
+      </c>
+      <c r="G39" s="23" t="s">
+        <v>160</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="I39" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="J39" s="9">
+        <v>124</v>
+      </c>
+      <c r="I39" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J39" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="L39" s="9">
         <v>1</v>
       </c>
-      <c r="K39" s="9"/>
-    </row>
-    <row r="40" spans="1:11" ht="24">
+      <c r="M39" s="9"/>
+    </row>
+    <row r="40" spans="1:13" ht="24.75" thickBot="1">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="I40" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="J40" s="11">
+        <v>166</v>
+      </c>
+      <c r="I40" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J40" s="27" t="s">
+        <v>289</v>
+      </c>
+      <c r="K40" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="L40" s="11">
         <v>1</v>
       </c>
-      <c r="K40" s="11"/>
-    </row>
-    <row r="41" spans="1:11">
+      <c r="M40" s="11"/>
+    </row>
+    <row r="41" spans="1:13" ht="15.75" thickBot="1">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="G41" s="10" t="s">
-        <v>250</v>
+        <v>127</v>
+      </c>
+      <c r="G41" s="23" t="s">
+        <v>236</v>
       </c>
       <c r="H41" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I41" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J41" s="9">
+      <c r="I41" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J41" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="L41" s="9">
         <v>2</v>
       </c>
-      <c r="K41" s="9"/>
-    </row>
-    <row r="42" spans="1:11">
+      <c r="M41" s="9"/>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" thickBot="1">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="H42" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I42" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J42" s="11">
+      <c r="I42" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="K42" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="L42" s="11">
         <v>1</v>
       </c>
-      <c r="K42" s="11"/>
-    </row>
-    <row r="43" spans="1:11">
+      <c r="M42" s="11"/>
+    </row>
+    <row r="43" spans="1:13" ht="15.75" thickBot="1">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>255</v>
+        <v>127</v>
+      </c>
+      <c r="G43" s="23" t="s">
+        <v>241</v>
       </c>
       <c r="H43" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I43" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="J43" s="9">
+      <c r="I43" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="L43" s="9">
         <v>4</v>
       </c>
-      <c r="K43" s="9"/>
-    </row>
-    <row r="44" spans="1:11" ht="24">
+      <c r="M43" s="9"/>
+    </row>
+    <row r="44" spans="1:13" ht="24.75" thickBot="1">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G44" s="12" t="s">
-        <v>252</v>
+        <v>127</v>
+      </c>
+      <c r="G44" s="25" t="s">
+        <v>238</v>
       </c>
       <c r="H44" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I44" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="J44" s="11">
+      <c r="I44" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J44" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="K44" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="L44" s="11">
         <v>11</v>
       </c>
-      <c r="K44" s="11"/>
-    </row>
-    <row r="45" spans="1:11" ht="24">
+      <c r="M44" s="11"/>
+    </row>
+    <row r="45" spans="1:13" ht="36.75" thickBot="1">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G45" s="10" t="s">
-        <v>190</v>
+      <c r="G45" s="23" t="s">
+        <v>179</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="I45" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="I45" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J45" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="K45" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J45" s="9">
+      <c r="L45" s="9">
         <v>1</v>
       </c>
-      <c r="K45" s="9"/>
-    </row>
-    <row r="46" spans="1:11">
+      <c r="M45" s="9"/>
+    </row>
+    <row r="46" spans="1:13" ht="15.75" thickBot="1">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="F46" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="G46" s="12" t="s">
-        <v>194</v>
+      <c r="G46" s="25" t="s">
+        <v>183</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="I46" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="I46" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J46" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="K46" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J46" s="11">
+      <c r="L46" s="11">
         <v>1</v>
       </c>
-      <c r="K46" s="11"/>
-    </row>
-    <row r="47" spans="1:11" ht="24">
+      <c r="M46" s="11"/>
+    </row>
+    <row r="47" spans="1:13" ht="24.75" thickBot="1">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="G47" s="10" t="s">
-        <v>200</v>
+        <v>188</v>
+      </c>
+      <c r="G47" s="23" t="s">
+        <v>189</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="I47" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="I47" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J47" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="K47" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J47" s="9">
+      <c r="L47" s="9">
         <v>1</v>
       </c>
-      <c r="K47" s="9"/>
-    </row>
-    <row r="48" spans="1:11" ht="36">
+      <c r="M47" s="9"/>
+    </row>
+    <row r="48" spans="1:13" ht="48.75" thickBot="1">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="G48" s="12" t="s">
-        <v>205</v>
+        <v>193</v>
+      </c>
+      <c r="G48" s="25" t="s">
+        <v>194</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="I48" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="I48" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J48" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="K48" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J48" s="11">
+      <c r="L48" s="11">
         <v>1</v>
       </c>
-      <c r="K48" s="11"/>
-    </row>
-    <row r="49" spans="1:11">
+      <c r="M48" s="11"/>
+    </row>
+    <row r="49" spans="1:13" ht="15.75" thickBot="1">
       <c r="A49" s="2"/>
       <c r="B49" s="7">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="C49" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="D49" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>207</v>
-      </c>
       <c r="E49" s="10" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="G49" s="10" t="s">
-        <v>210</v>
+        <v>198</v>
+      </c>
+      <c r="G49" s="23" t="s">
+        <v>199</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="I49" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="I49" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="K49" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J49" s="9">
+      <c r="L49" s="9">
         <v>1</v>
       </c>
-      <c r="K49" s="9"/>
-    </row>
-    <row r="50" spans="1:11">
+      <c r="M49" s="9"/>
+    </row>
+    <row r="50" spans="1:13" ht="15.75" thickBot="1">
       <c r="A50" s="2"/>
       <c r="B50" s="7">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="I50" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="I50" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="K50" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J50" s="11">
+      <c r="L50" s="11">
         <v>1</v>
       </c>
-      <c r="K50" s="11"/>
-    </row>
-    <row r="51" spans="1:11" ht="48">
+      <c r="M50" s="11"/>
+    </row>
+    <row r="51" spans="1:13" ht="48.75" thickBot="1">
       <c r="A51" s="2"/>
       <c r="B51" s="7">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>218</v>
+        <v>206</v>
+      </c>
+      <c r="G51" s="23" t="s">
+        <v>207</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="I51" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="I51" s="26" t="s">
+        <v>300</v>
+      </c>
+      <c r="J51" s="30" t="s">
+        <v>301</v>
+      </c>
+      <c r="K51" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J51" s="9">
+      <c r="L51" s="9">
         <v>1</v>
       </c>
-      <c r="K51" s="9"/>
-    </row>
-    <row r="52" spans="1:11" ht="24">
+      <c r="M51" s="9"/>
+    </row>
+    <row r="52" spans="1:13" ht="24.75" thickBot="1">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>221</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>222</v>
+        <v>210</v>
+      </c>
+      <c r="G52" s="25" t="s">
+        <v>211</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="I52" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="I52" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="K52" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J52" s="11">
+      <c r="L52" s="11">
         <v>1</v>
       </c>
-      <c r="K52" s="11"/>
-    </row>
-    <row r="53" spans="1:11">
+      <c r="M52" s="11"/>
+    </row>
+    <row r="53" spans="1:13" ht="15.75" thickBot="1">
       <c r="A53" s="2"/>
       <c r="B53" s="7">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>227</v>
+        <v>215</v>
+      </c>
+      <c r="G53" s="23" t="s">
+        <v>216</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="I53" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="I53" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="K53" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J53" s="9">
+      <c r="L53" s="9">
         <v>1</v>
       </c>
-      <c r="K53" s="9"/>
-    </row>
-    <row r="54" spans="1:11">
+      <c r="M53" s="9"/>
+    </row>
+    <row r="54" spans="1:13" ht="15.75" thickBot="1">
       <c r="A54" s="2"/>
       <c r="B54" s="7">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="G54" s="12" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="H54" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="I54" s="12" t="s">
+      <c r="I54" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J54" s="19" t="s">
+        <v>304</v>
+      </c>
+      <c r="K54" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J54" s="11">
+      <c r="L54" s="11">
         <v>1</v>
       </c>
-      <c r="K54" s="11"/>
+      <c r="M54" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>